<commit_message>
Harness box bench: SBU1 from a low-impedance source; FMD-033 SPICE note
The 1 kOhm series resistor on the SBU1 bench source divided against the box's
R2+R3 (240 Ohm) to 0.97 V: no intercept on an intact box and no threshold sweep
above 1 V. WP-H-06 0.12 §3.1, checklist 0.3 (plus a load check) and the bench
wiring drawing now use a low-impedance source, current-limited to about 50 mA.
WP-H-02 0.12 HE-08: the device's SBU1 driver must source about 21 mA.
FMEDA SG-009 0.8: FMD-033 note with the SPICE pilot's per-path predictions;
classification unchanged. Found by the harness box SPICE pilot (PR #510).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="362">
   <si>
     <t xml:space="preserve">FMEDA — SG-009 stock AEB availability (relay and forwarding path), generic failure rates</t>
   </si>
@@ -52,120 +52,129 @@
     <t xml:space="preserve">Revision</t>
   </si>
   <si>
+    <t xml:space="preserve">0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-07 ASIL B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LD-HARA-001 goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude (AI-assisted draft)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description of change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stub without components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.7</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-07 ASIL B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LD-HARA-001 goal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Author</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude (AI-assisted draft)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description of change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stub without components</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
-  </si>
-  <si>
     <t xml:space="preserve">Format review: target as data, rate kind and wire ends as fields; no rate, classification or metric change</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FMD-033 note: harness box SPICE pilot predictions per short path (PR #510); whole mode stays single-point; no rate, classification or metric change</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mission profile</t>
   </si>
   <si>
@@ -835,7 +844,7 @@
     <t xml:space="preserve">DFM-021</t>
   </si>
   <si>
-    <t xml:space="preserve">Car or camera bus loaded in either switch state (RR-2026-010 F-07)</t>
+    <t xml:space="preserve">Car or camera bus loaded in either switch state (RR-2026-010 F-07). The harness box SPICE pilot (PR #510; idealised model, generic transceivers; a prediction, no credit) splits the mode: a lower-diode short to GND on CAN_H loses dominant bits; an upper-diode short to VIN holds the line near 13 V, outside the receiver common-mode range; CAN_L to GND and 1 kOhm leakage leave readable levels. A D3 short on camera CAN_H to GND also stops the joined stock bus in pass-through. The whole mode stays single-point until VS-HW-24 (d) measures the split on a real box</t>
   </si>
   <si>
     <t xml:space="preserve">FMD-034</t>
@@ -1617,30 +1626,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!O2:O35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
@@ -1654,7 +1663,7 @@
         <v>PASS</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -1688,33 +1697,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>7</v>
@@ -1760,7 +1769,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">07_SPFM_Calculation!D2</f>
@@ -1791,10 +1800,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>7</v>
@@ -1802,200 +1811,200 @@
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>320</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -2022,58 +2031,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>358</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>355</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -2092,7 +2101,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100"/>
@@ -2198,7 +2207,7 @@
     </row>
     <row r="8" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>41</v>
@@ -2207,7 +2216,21 @@
         <v>16</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -2235,42 +2258,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2308,469 +2331,469 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>100</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L14" s="3"/>
     </row>
@@ -2804,136 +2827,136 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2964,87 +2987,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>40</v>
@@ -3054,19 +3077,19 @@
         <v>20</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="N2" s="3" t="n">
         <f aca="false">IF(D2="No",0,IF(AND(I2="No",J2="No"),H2,0))</f>
@@ -3089,31 +3112,31 @@
         <v>RF</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>5</v>
@@ -3123,10 +3146,10 @@
         <v>2.5</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="n">
@@ -3154,31 +3177,31 @@
         <v>SPF</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>55</v>
@@ -3188,10 +3211,10 @@
         <v>27.5</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="n">
@@ -3224,22 +3247,22 @@
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>80</v>
@@ -3249,19 +3272,19 @@
         <v>16</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N5" s="3" t="n">
         <f aca="false">IF(D5="No",0,IF(AND(I5="No",J5="No"),H5,0))</f>
@@ -3284,29 +3307,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>10</v>
@@ -3316,19 +3339,19 @@
         <v>2</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="N6" s="3" t="n">
         <f aca="false">IF(D6="No",0,IF(AND(I6="No",J6="No"),H6,0))</f>
@@ -3351,29 +3374,29 @@
         <v>RF</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>10</v>
@@ -3383,19 +3406,19 @@
         <v>2</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="L7" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N7" s="3" t="n">
         <f aca="false">IF(D7="No",0,IF(AND(I7="No",J7="No"),H7,0))</f>
@@ -3418,31 +3441,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>90</v>
@@ -3452,19 +3475,19 @@
         <v>90</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N8" s="3" t="n">
         <f aca="false">IF(D8="No",0,IF(AND(I8="No",J8="No"),H8,0))</f>
@@ -3487,29 +3510,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>5</v>
@@ -3519,19 +3542,19 @@
         <v>5</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="N9" s="3" t="n">
         <f aca="false">IF(D9="No",0,IF(AND(I9="No",J9="No"),H9,0))</f>
@@ -3554,29 +3577,29 @@
         <v>RF</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>5</v>
@@ -3586,10 +3609,10 @@
         <v>5</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="n">
@@ -3617,31 +3640,31 @@
         <v>Safe</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>50</v>
@@ -3651,19 +3674,19 @@
         <v>5</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="L11" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N11" s="3" t="n">
         <f aca="false">IF(D11="No",0,IF(AND(I11="No",J11="No"),H11,0))</f>
@@ -3686,31 +3709,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>10</v>
@@ -3720,10 +3743,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3" t="n">
@@ -3751,29 +3774,29 @@
         <v>SPF</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>40</v>
@@ -3783,10 +3806,10 @@
         <v>4</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K13" s="3"/>
       <c r="L13" s="3" t="n">
@@ -3814,29 +3837,29 @@
         <v>Safe</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>50</v>
@@ -3846,10 +3869,10 @@
         <v>7.5</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3" t="n">
@@ -3877,31 +3900,31 @@
         <v>Safe</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="T14" s="3"/>
       <c r="U14" s="3" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>30</v>
@@ -3911,19 +3934,19 @@
         <v>4.5</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>60</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="N15" s="3" t="n">
         <f aca="false">IF(D15="No",0,IF(AND(I15="No",J15="No"),H15,0))</f>
@@ -3946,31 +3969,31 @@
         <v>RF</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="T15" s="3"/>
       <c r="U15" s="3" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>20</v>
@@ -3980,10 +4003,10 @@
         <v>3</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K16" s="3"/>
       <c r="L16" s="3" t="n">
@@ -4011,29 +4034,29 @@
         <v>Safe</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>30</v>
@@ -4043,10 +4066,10 @@
         <v>6</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="n">
@@ -4074,31 +4097,31 @@
         <v>SPF</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="T17" s="3"/>
       <c r="U17" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>30</v>
@@ -4108,10 +4131,10 @@
         <v>6</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="3" t="n">
@@ -4139,31 +4162,31 @@
         <v>SPF</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="T18" s="3"/>
       <c r="U18" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>40</v>
@@ -4173,10 +4196,10 @@
         <v>8</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3" t="n">
@@ -4209,22 +4232,22 @@
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>30</v>
@@ -4234,10 +4257,10 @@
         <v>15</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="3" t="n">
@@ -4265,31 +4288,31 @@
         <v>SPF</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="T20" s="3"/>
       <c r="U20" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>30</v>
@@ -4299,10 +4322,10 @@
         <v>15</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="3" t="n">
@@ -4330,31 +4353,31 @@
         <v>Safe</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="T21" s="3"/>
       <c r="U21" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C22" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>40</v>
@@ -4364,10 +4387,10 @@
         <v>20</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="3" t="n">
@@ -4395,31 +4418,31 @@
         <v>SPF</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="T22" s="3"/>
       <c r="U22" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C23" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>50</v>
@@ -4429,10 +4452,10 @@
         <v>2.5</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="3" t="n">
@@ -4460,31 +4483,31 @@
         <v>SPF</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="T23" s="3"/>
       <c r="U23" s="3" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>50</v>
@@ -4494,10 +4517,10 @@
         <v>2.5</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="3" t="n">
@@ -4525,31 +4548,31 @@
         <v>Safe</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="T24" s="3"/>
       <c r="U24" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>60</v>
@@ -4559,10 +4582,10 @@
         <v>0.24</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3" t="n">
@@ -4590,31 +4613,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="T25" s="3"/>
       <c r="U25" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>40</v>
@@ -4624,10 +4647,10 @@
         <v>0.16</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="3" t="n">
@@ -4655,31 +4678,31 @@
         <v>Safe</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="T26" s="3"/>
       <c r="U26" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>40</v>
@@ -4689,10 +4712,10 @@
         <v>1.2</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3" t="n">
@@ -4720,31 +4743,31 @@
         <v>SPF</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="T27" s="3"/>
       <c r="U27" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>20</v>
@@ -4754,10 +4777,10 @@
         <v>0.6</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3" t="n">
@@ -4785,31 +4808,31 @@
         <v>SPF</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="T28" s="3"/>
       <c r="U28" s="3" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>40</v>
@@ -4819,10 +4842,10 @@
         <v>1.2</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="n">
@@ -4850,31 +4873,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="T29" s="3"/>
       <c r="U29" s="3" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>30</v>
@@ -4884,10 +4907,10 @@
         <v>0.6</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="n">
@@ -4915,31 +4938,31 @@
         <v>SPF</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="T30" s="3"/>
       <c r="U30" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>70</v>
@@ -4949,10 +4972,10 @@
         <v>1.4</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3" t="n">
@@ -4980,31 +5003,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="T31" s="3"/>
       <c r="U31" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C32" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>30</v>
@@ -5014,10 +5037,10 @@
         <v>3</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="3" t="n">
@@ -5045,31 +5068,31 @@
         <v>SPF</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="T32" s="3"/>
       <c r="U32" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C33" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>70</v>
@@ -5079,10 +5102,10 @@
         <v>7</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="3" t="n">
@@ -5110,31 +5133,31 @@
         <v>Safe</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="T33" s="3"/>
       <c r="U33" s="3" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>50</v>
@@ -5144,10 +5167,10 @@
         <v>1</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3" t="n">
@@ -5175,31 +5198,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="T34" s="3"/>
       <c r="U34" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>50</v>
@@ -5209,10 +5232,10 @@
         <v>1</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3" t="n">
@@ -5240,11 +5263,11 @@
         <v>Safe</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="T35" s="3"/>
       <c r="U35" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -5271,57 +5294,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -5351,22 +5374,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5374,10 +5397,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!O2:O35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
@@ -5426,22 +5449,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>299</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>296</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5449,10 +5472,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!Q2:Q35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$O$2:$O$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$G$2:$G$2))</f>

</xml_diff>

<commit_message>
FMEDA SG-009 rev 0.9: camera-side termination R7/R8
FMD-C-014 (2 x 120 Ohm, generic 0.4 FIT): one resistor open is latent (both
open leave the camera bus unterminated in intercept, per the SPICE pilot and
VS-HW-24 (e)); a short is single-point for SG-07 (camera frames lost while the
device forwards). SG-07: 288 FIT, SPFM 78.1 %, LFM 97.6 %, lambda SPF+RF
63.1 FIT. Planned-measure chain 83.6 -> 87.3 -> 94.5 %, still meets B.
WP-H-03 0.10, WP-H-04 0.12, fmea-plan v0.36, what-if test updated.
No DFMEA row yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="378">
   <si>
     <t xml:space="preserve">FMEDA — SG-009 stock AEB availability (relay and forwarding path), generic failure rates</t>
   </si>
@@ -52,129 +52,135 @@
     <t xml:space="preserve">Revision</t>
   </si>
   <si>
+    <t xml:space="preserve">0.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-07 ASIL B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LD-HARA-001 goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude (AI-assisted draft)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description of change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stub without components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format review: target as data, rate kind and wire ends as fields; no rate, classification or metric change</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.8</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-07 ASIL B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LD-HARA-001 goal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Author</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude (AI-assisted draft)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description of change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stub without components</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format review: target as data, rate kind and wire ends as fields; no rate, classification or metric change</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-10-27</t>
   </si>
   <si>
     <t xml:space="preserve">FMD-033 note: harness box SPICE pilot predictions per short path (PR #510); whole mode stays single-point; no rate, classification or metric change</t>
   </si>
   <si>
+    <t xml:space="preserve">Camera-side termination R7/R8 added (FMD-C-014): one open latent, short single-point; total and SPF rates change</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mission profile</t>
   </si>
   <si>
@@ -184,7 +190,7 @@
     <t xml:space="preserve">FIT source</t>
   </si>
   <si>
-    <t xml:space="preserve">13 components: 12 generic, 1 handbook; 0 converted to the mission profile (IEC 61709). Handbook set approved by the lead (WP-H-03 §2.3, DQ-068); per-part source in 03_HW_Element_Catalog. Generic rates are order-of-magnitude estimates, not evidence</t>
+    <t xml:space="preserve">14 components: 13 generic, 1 handbook; 0 converted to the mission profile (IEC 61709). Handbook set approved by the lead (WP-H-03 §2.3, DQ-068); per-part source in 03_HW_Element_Catalog. Generic rates are order-of-magnitude estimates, not evidence</t>
   </si>
   <si>
     <t xml:space="preserve">Environmental class</t>
@@ -385,6 +391,18 @@
     <t xml:space="preserve">Generic estimate (small-signal Schottky diode array BAS40SDW, 2 × about 1 FIT). The part is known from the harness box v3 drawing (RR-2026-010 HB-01..HB-06) and maps to the SN 29500 discrete-semiconductor class, but no reference value could be obtained: the standard and the vendor FIT reports were not reachable from the analysis environment (2026-10-16). Stays generic until the safety manager confirms the source (WP-H-03 OI-2) and the value is looked up; shipped parts unconfirmed (VS-HW-02)</t>
   </si>
   <si>
+    <t xml:space="preserve">FMD-C-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camera-side termination in intercept: 2 × 120 Ω thick-film resistor (R7, and R8 through the harness P13–P15 loopback), 60 Ω together</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7, R8 (harness box)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic estimate (SMD thick-film chip resistor, 2 × about 0.2 FIT), as FMD-C-011. Part class known from the harness box v3 drawing (RR-2026-010 HB-05); maps to the SN 29500 passive-component class, but no reference value could be obtained (standard not reachable, 2026-10-16). Stays generic until the source is confirmed (WP-H-03 OI-2); shipped parts unconfirmed (VS-HW-02)</t>
+  </si>
+  <si>
     <t xml:space="preserve">FMD-C-008</t>
   </si>
   <si>
@@ -856,6 +874,24 @@
     <t xml:space="preserve">Latent loss of bus protection</t>
   </si>
   <si>
+    <t xml:space="preserve">FMD-035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One resistor open (camera side left with 120 Ω in intercept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latent: violates SG-009 only with the second resistor open (or the loopback open), which leaves the camera bus unterminated in intercept: the harness box SPICE pilot predicts a recessive edge of about 10.5 µs, missing the 1.5 µs sample point, so camera frames are lost while the device forwards (spice/predictions.md T-both-open, a prediction, no credit). One open alone leaves 120 Ω and an edge of about 0.06 µs. No check in the field; VS-HW-24 (e) measures both cases. Pass-through is not affected (R7/R8 sit on the NO side). No DFMEA row yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FMD-036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short (camera CAN2_H to CAN2_L in intercept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camera bus held recessive in intercept: no camera frames reach the device, so stock PCS messages are not forwarded. RX checks cover car-side messages only (as FMD-017), so no mechanism is credited. Pass-through is not affected (R7/R8 sit on the NO side). No DFMEA row yet</t>
+  </si>
+  <si>
     <t xml:space="preserve">FMD-023</t>
   </si>
   <si>
@@ -1063,28 +1099,40 @@
     <t xml:space="preserve">OI-14</t>
   </si>
   <si>
+    <t xml:space="preserve">FMD-035 (FMD-C-014): latent fault without coverage: One resistor open (camera side left with 120 Ω in intercept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FMD-036 (FMD-C-014): single-point fault without a safety mechanism: Short (camera CAN2_H to CAN2_L in intercept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-16</t>
+  </si>
+  <si>
     <t xml:space="preserve">FMD-023 (FMD-C-008): single-point fault without a safety mechanism: Open in the stock camera path</t>
   </si>
   <si>
-    <t xml:space="preserve">OI-15</t>
+    <t xml:space="preserve">OI-17</t>
   </si>
   <si>
     <t xml:space="preserve">FMD-025 (FMD-C-009): latent fault without coverage: Watchdog does not expire (LSI stopped, IWDG fault)</t>
   </si>
   <si>
-    <t xml:space="preserve">OI-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 of 13 failure rates are generic estimates: replace with handbook or supplier values per part (WP-H-03 §2.3, OI-10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-17</t>
+    <t xml:space="preserve">OI-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 of 14 failure rates are generic estimates: replace with handbook or supplier values per part (WP-H-03 §2.3, OI-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-19</t>
   </si>
   <si>
     <t xml:space="preserve">No rate is converted to the mission profile (IEC 61709)</t>
   </si>
   <si>
-    <t xml:space="preserve">OI-18</t>
+    <t xml:space="preserve">OI-20</t>
   </si>
   <si>
     <t xml:space="preserve">Dual-point PMHF term not computed</t>
@@ -1626,34 +1674,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="C2" s="0" t="n">
-        <f aca="false">SUM(06_FMEDA_Worksheet!O2:O35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
-        <v>62.9</v>
+        <f aca="false">SUM(06_FMEDA_Worksheet!O2:O37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
+        <v>63.06</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>100</v>
@@ -1663,7 +1711,7 @@
         <v>PASS</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -1697,33 +1745,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>7</v>
@@ -1740,7 +1788,7 @@
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">07_SPFM_Calculation!E2</f>
-        <v>0.781141266527488</v>
+        <v>0.780889506601807</v>
       </c>
       <c r="D4" s="0" t="n">
         <f aca="false">07_SPFM_Calculation!F2</f>
@@ -1748,7 +1796,7 @@
       </c>
       <c r="E4" s="0" t="n">
         <f aca="false">08_LFM_Calculation!E2</f>
-        <v>0.97706013363029</v>
+        <v>0.976016730444069</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">08_LFM_Calculation!F2</f>
@@ -1756,7 +1804,7 @@
       </c>
       <c r="G4" s="0" t="n">
         <f aca="false">09_PMHF_Calculation!C2</f>
-        <v>62.9</v>
+        <v>63.06</v>
       </c>
       <c r="H4" s="0" t="n">
         <f aca="false">09_PMHF_Calculation!D2</f>
@@ -1769,11 +1817,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">07_SPFM_Calculation!D2</f>
-        <v>287.4</v>
+        <v>287.8</v>
       </c>
     </row>
   </sheetData>
@@ -1792,7 +1840,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
@@ -1800,10 +1848,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>7</v>
@@ -1811,200 +1859,222 @@
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>329</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>364</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>366</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -2031,58 +2101,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -2101,7 +2171,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100"/>
@@ -2221,16 +2291,30 @@
     </row>
     <row r="9" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>46</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2258,42 +2342,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2396,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -2331,471 +2415,503 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>100</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K13" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K14" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="L14" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L15" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2827,136 +2943,136 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2975,7 +3091,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:U37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
@@ -2987,87 +3103,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>40</v>
@@ -3077,19 +3193,19 @@
         <v>20</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="N2" s="3" t="n">
         <f aca="false">IF(D2="No",0,IF(AND(I2="No",J2="No"),H2,0))</f>
@@ -3112,31 +3228,31 @@
         <v>RF</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>5</v>
@@ -3146,10 +3262,10 @@
         <v>2.5</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="n">
@@ -3177,31 +3293,31 @@
         <v>SPF</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>55</v>
@@ -3211,10 +3327,10 @@
         <v>27.5</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="n">
@@ -3247,22 +3363,22 @@
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>80</v>
@@ -3272,19 +3388,19 @@
         <v>16</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="N5" s="3" t="n">
         <f aca="false">IF(D5="No",0,IF(AND(I5="No",J5="No"),H5,0))</f>
@@ -3307,29 +3423,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>10</v>
@@ -3339,19 +3455,19 @@
         <v>2</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="N6" s="3" t="n">
         <f aca="false">IF(D6="No",0,IF(AND(I6="No",J6="No"),H6,0))</f>
@@ -3374,29 +3490,29 @@
         <v>RF</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>10</v>
@@ -3406,19 +3522,19 @@
         <v>2</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="L7" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="N7" s="3" t="n">
         <f aca="false">IF(D7="No",0,IF(AND(I7="No",J7="No"),H7,0))</f>
@@ -3441,31 +3557,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>90</v>
@@ -3475,19 +3591,19 @@
         <v>90</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="N8" s="3" t="n">
         <f aca="false">IF(D8="No",0,IF(AND(I8="No",J8="No"),H8,0))</f>
@@ -3510,29 +3626,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>5</v>
@@ -3542,19 +3658,19 @@
         <v>5</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="N9" s="3" t="n">
         <f aca="false">IF(D9="No",0,IF(AND(I9="No",J9="No"),H9,0))</f>
@@ -3577,29 +3693,29 @@
         <v>RF</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>5</v>
@@ -3609,10 +3725,10 @@
         <v>5</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="n">
@@ -3640,31 +3756,31 @@
         <v>Safe</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>50</v>
@@ -3674,19 +3790,19 @@
         <v>5</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="L11" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="N11" s="3" t="n">
         <f aca="false">IF(D11="No",0,IF(AND(I11="No",J11="No"),H11,0))</f>
@@ -3709,31 +3825,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>10</v>
@@ -3743,10 +3859,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3" t="n">
@@ -3774,29 +3890,29 @@
         <v>SPF</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>40</v>
@@ -3806,10 +3922,10 @@
         <v>4</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K13" s="3"/>
       <c r="L13" s="3" t="n">
@@ -3837,29 +3953,29 @@
         <v>Safe</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>50</v>
@@ -3869,10 +3985,10 @@
         <v>7.5</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3" t="n">
@@ -3900,31 +4016,31 @@
         <v>Safe</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="T14" s="3"/>
       <c r="U14" s="3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>30</v>
@@ -3934,19 +4050,19 @@
         <v>4.5</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>60</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="N15" s="3" t="n">
         <f aca="false">IF(D15="No",0,IF(AND(I15="No",J15="No"),H15,0))</f>
@@ -3969,31 +4085,31 @@
         <v>RF</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="T15" s="3"/>
       <c r="U15" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>20</v>
@@ -4003,10 +4119,10 @@
         <v>3</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K16" s="3"/>
       <c r="L16" s="3" t="n">
@@ -4034,29 +4150,29 @@
         <v>Safe</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>30</v>
@@ -4066,10 +4182,10 @@
         <v>6</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="n">
@@ -4097,31 +4213,31 @@
         <v>SPF</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="T17" s="3"/>
       <c r="U17" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>30</v>
@@ -4131,10 +4247,10 @@
         <v>6</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="3" t="n">
@@ -4162,31 +4278,31 @@
         <v>SPF</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="T18" s="3"/>
       <c r="U18" s="3" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>40</v>
@@ -4196,10 +4312,10 @@
         <v>8</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3" t="n">
@@ -4232,22 +4348,22 @@
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>30</v>
@@ -4257,10 +4373,10 @@
         <v>15</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="3" t="n">
@@ -4288,31 +4404,31 @@
         <v>SPF</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="T20" s="3"/>
       <c r="U20" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>30</v>
@@ -4322,10 +4438,10 @@
         <v>15</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="3" t="n">
@@ -4353,31 +4469,31 @@
         <v>Safe</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="T21" s="3"/>
       <c r="U21" s="3" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C22" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>40</v>
@@ -4387,10 +4503,10 @@
         <v>20</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="3" t="n">
@@ -4418,31 +4534,31 @@
         <v>SPF</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="T22" s="3"/>
       <c r="U22" s="3" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C23" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>50</v>
@@ -4452,10 +4568,10 @@
         <v>2.5</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="3" t="n">
@@ -4483,31 +4599,31 @@
         <v>SPF</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="T23" s="3"/>
       <c r="U23" s="3" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>50</v>
@@ -4517,10 +4633,10 @@
         <v>2.5</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="3" t="n">
@@ -4548,31 +4664,31 @@
         <v>Safe</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="T24" s="3"/>
       <c r="U24" s="3" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>60</v>
@@ -4582,10 +4698,10 @@
         <v>0.24</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3" t="n">
@@ -4613,31 +4729,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="T25" s="3"/>
       <c r="U25" s="3" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>40</v>
@@ -4647,10 +4763,10 @@
         <v>0.16</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="3" t="n">
@@ -4678,31 +4794,31 @@
         <v>Safe</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="T26" s="3"/>
       <c r="U26" s="3" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>40</v>
@@ -4712,10 +4828,10 @@
         <v>1.2</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3" t="n">
@@ -4743,31 +4859,31 @@
         <v>SPF</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="T27" s="3"/>
       <c r="U27" s="3" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>20</v>
@@ -4777,10 +4893,10 @@
         <v>0.6</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3" t="n">
@@ -4808,31 +4924,31 @@
         <v>SPF</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="T28" s="3"/>
       <c r="U28" s="3" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>40</v>
@@ -4842,10 +4958,10 @@
         <v>1.2</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="n">
@@ -4873,31 +4989,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="T29" s="3"/>
       <c r="U29" s="3" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>30</v>
@@ -4907,10 +5023,10 @@
         <v>0.6</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="n">
@@ -4938,31 +5054,31 @@
         <v>SPF</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="T30" s="3"/>
       <c r="U30" s="3" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>70</v>
@@ -4972,10 +5088,10 @@
         <v>1.4</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3" t="n">
@@ -5003,44 +5119,44 @@
         <v>MPF_L</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="T31" s="3"/>
       <c r="U31" s="3" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H32" s="3" t="n">
         <f aca="false">C32*G32/100</f>
-        <v>3</v>
+        <v>0.24</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="3" t="n">
@@ -5053,7 +5169,7 @@
       </c>
       <c r="O32" s="3" t="n">
         <f aca="false">IF(D32="No",0,IF(AND(I32="Yes",L32=0),H32,0))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P32" s="3" t="n">
         <f aca="false">IF(D32="No",0,IF(AND(I32="Yes",L32&gt;0),H32*(1-L32/100),0))</f>
@@ -5061,51 +5177,49 @@
       </c>
       <c r="Q32" s="3" t="n">
         <f aca="false">IF(D32="No",0,IF(AND(I32="No",J32="Yes"),H32*(1-L32/100),0))</f>
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="R32" s="3" t="str">
         <f aca="false">IF(D32="No","Safe",IF(I32="Yes",IF(L32=0,"SPF","RF"),IF(J32="Yes",IF(L32=0,"MPF_L","MPF_D"),"Safe")))</f>
-        <v>SPF</v>
-      </c>
-      <c r="S32" s="3" t="s">
-        <v>243</v>
-      </c>
+        <v>MPF_L</v>
+      </c>
+      <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H33" s="3" t="n">
         <f aca="false">C33*G33/100</f>
-        <v>7</v>
+        <v>0.16</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="3" t="n">
@@ -5114,11 +5228,11 @@
       <c r="M33" s="3"/>
       <c r="N33" s="3" t="n">
         <f aca="false">IF(D33="No",0,IF(AND(I33="No",J33="No"),H33,0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O33" s="3" t="n">
         <f aca="false">IF(D33="No",0,IF(AND(I33="Yes",L33=0),H33,0))</f>
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="P33" s="3" t="n">
         <f aca="false">IF(D33="No",0,IF(AND(I33="Yes",L33&gt;0),H33*(1-L33/100),0))</f>
@@ -5130,47 +5244,45 @@
       </c>
       <c r="R33" s="3" t="str">
         <f aca="false">IF(D33="No","Safe",IF(I33="Yes",IF(L33=0,"SPF","RF"),IF(J33="Yes",IF(L33=0,"MPF_L","MPF_D"),"Safe")))</f>
-        <v>Safe</v>
-      </c>
-      <c r="S33" s="3" t="s">
-        <v>279</v>
-      </c>
+        <v>SPF</v>
+      </c>
+      <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H34" s="3" t="n">
         <f aca="false">C34*G34/100</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3" t="n">
@@ -5183,7 +5295,7 @@
       </c>
       <c r="O34" s="3" t="n">
         <f aca="false">IF(D34="No",0,IF(AND(I34="Yes",L34=0),H34,0))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P34" s="3" t="n">
         <f aca="false">IF(D34="No",0,IF(AND(I34="Yes",L34&gt;0),H34*(1-L34/100),0))</f>
@@ -5191,51 +5303,51 @@
       </c>
       <c r="Q34" s="3" t="n">
         <f aca="false">IF(D34="No",0,IF(AND(I34="No",J34="Yes"),H34*(1-L34/100),0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R34" s="3" t="str">
         <f aca="false">IF(D34="No","Safe",IF(I34="Yes",IF(L34=0,"SPF","RF"),IF(J34="Yes",IF(L34=0,"MPF_L","MPF_D"),"Safe")))</f>
-        <v>MPF_L</v>
+        <v>SPF</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>283</v>
+        <v>249</v>
       </c>
       <c r="T34" s="3"/>
       <c r="U34" s="3" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="H35" s="3" t="n">
         <f aca="false">C35*G35/100</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3" t="n">
@@ -5244,7 +5356,7 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3" t="n">
         <f aca="false">IF(D35="No",0,IF(AND(I35="No",J35="No"),H35,0))</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O35" s="3" t="n">
         <f aca="false">IF(D35="No",0,IF(AND(I35="Yes",L35=0),H35,0))</f>
@@ -5263,11 +5375,141 @@
         <v>Safe</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="T35" s="3"/>
       <c r="U35" s="3" t="s">
-        <v>287</v>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <f aca="false">C36*G36/100</f>
+        <v>1</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3" t="n">
+        <f aca="false">IF(D36="No",0,IF(AND(I36="No",J36="No"),H36,0))</f>
+        <v>0</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <f aca="false">IF(D36="No",0,IF(AND(I36="Yes",L36=0),H36,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P36" s="3" t="n">
+        <f aca="false">IF(D36="No",0,IF(AND(I36="Yes",L36&gt;0),H36*(1-L36/100),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3" t="n">
+        <f aca="false">IF(D36="No",0,IF(AND(I36="No",J36="Yes"),H36*(1-L36/100),0))</f>
+        <v>1</v>
+      </c>
+      <c r="R36" s="3" t="str">
+        <f aca="false">IF(D36="No","Safe",IF(I36="Yes",IF(L36=0,"SPF","RF"),IF(J36="Yes",IF(L36=0,"MPF_L","MPF_D"),"Safe")))</f>
+        <v>MPF_L</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="T36" s="3"/>
+      <c r="U36" s="3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <f aca="false">C37*G37/100</f>
+        <v>1</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3" t="n">
+        <f aca="false">IF(D37="No",0,IF(AND(I37="No",J37="No"),H37,0))</f>
+        <v>1</v>
+      </c>
+      <c r="O37" s="3" t="n">
+        <f aca="false">IF(D37="No",0,IF(AND(I37="Yes",L37=0),H37,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <f aca="false">IF(D37="No",0,IF(AND(I37="Yes",L37&gt;0),H37*(1-L37/100),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="3" t="n">
+        <f aca="false">IF(D37="No",0,IF(AND(I37="No",J37="Yes"),H37*(1-L37/100),0))</f>
+        <v>0</v>
+      </c>
+      <c r="R37" s="3" t="str">
+        <f aca="false">IF(D37="No","Safe",IF(I37="Yes",IF(L37=0,"SPF","RF"),IF(J37="Yes",IF(L37=0,"MPF_L","MPF_D"),"Safe")))</f>
+        <v>Safe</v>
+      </c>
+      <c r="S37" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="T37" s="3"/>
+      <c r="U37" s="3" t="s">
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -5294,57 +5536,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -5374,22 +5616,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5397,22 +5639,22 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="C2" s="0" t="n">
-        <f aca="false">SUM(06_FMEDA_Worksheet!O2:O35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
-        <v>62.9</v>
+        <f aca="false">SUM(06_FMEDA_Worksheet!O2:O37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
+        <v>63.06</v>
       </c>
       <c r="D2" s="0" t="n">
-        <f aca="false">SUMIF(06_FMEDA_Worksheet!D2:D35,"Yes",06_FMEDA_Worksheet!H2:H35)</f>
-        <v>287.4</v>
+        <f aca="false">SUMIF(06_FMEDA_Worksheet!D2:D37,"Yes",06_FMEDA_Worksheet!H2:H37)</f>
+        <v>287.8</v>
       </c>
       <c r="E2" s="0" t="n">
         <f aca="false">1-C2/D2</f>
-        <v>0.781141266527488</v>
+        <v>0.780889506601807</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>0.9</v>
@@ -5449,22 +5691,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5472,22 +5714,22 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="C2" s="0" t="n">
-        <f aca="false">SUM(06_FMEDA_Worksheet!Q2:Q35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$O$2:$O$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$G$2:$G$2))</f>
-        <v>5.15</v>
+        <f aca="false">SUM(06_FMEDA_Worksheet!Q2:Q37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$O$2:$O$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$G$2:$G$2))</f>
+        <v>5.39</v>
       </c>
       <c r="D2" s="0" t="n">
-        <f aca="false">SUMIF(06_FMEDA_Worksheet!D2:D35,"Yes",06_FMEDA_Worksheet!H2:H35)-(SUM(06_FMEDA_Worksheet!O2:O35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P35)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2)))</f>
-        <v>224.5</v>
+        <f aca="false">SUMIF(06_FMEDA_Worksheet!D2:D37,"Yes",06_FMEDA_Worksheet!H2:H37)-(SUM(06_FMEDA_Worksheet!O2:O37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2)))</f>
+        <v>224.74</v>
       </c>
       <c r="E2" s="0" t="n">
         <f aca="false">IF(D2=0,1,1-C2/D2)</f>
-        <v>0.97706013363029</v>
+        <v>0.976016730444069</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>0.6</v>

</xml_diff>

<commit_message>
FMEDA SG-009 rev 0.10: link FMD-035/036 to DFMEA DFM-022/023
No rate, classification or metric change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/fmeda-sg009-review.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="382">
   <si>
     <t xml:space="preserve">FMEDA — SG-009 stock AEB availability (relay and forwarding path), generic failure rates</t>
   </si>
@@ -52,135 +52,141 @@
     <t xml:space="preserve">Revision</t>
   </si>
   <si>
+    <t xml:space="preserve">0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-07 ASIL B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LD-HARA-001 goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude (AI-assisted draft)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description of change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stub without components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format review: target as data, rate kind and wire ends as fields; no rate, classification or metric change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FMD-033 note: harness box SPICE pilot predictions per short path (PR #510); whole mode stays single-point; no rate, classification or metric change</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.9</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Targets (WP-H-04 §4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-07 ASIL B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LD-HARA-001 goal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG-009 ASIL B (reference only; the targets above are used)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Author</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude (AI-assisted draft)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jherrod Thomas (project maintainer); not yet reviewed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">assurance/08-analyses/fmea/analyses/fmeda-sg009.yaml (generated by tools/safety/export_fmeda_xlsx.py; do not edit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random hardware faults of the panda section and harness that can keep the stock camera's PCS messages from reaching the car (LD-HARA-001 SG-009, ASIL B; assurance WP-C-03 SG-07, ASIL B). Reference device at BL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description of change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stub without components</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First quantitative FMEDA at BL-002 with generic failure rates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relay re-based to the harness box v3 analog switches U1/U2 and its pull-down, supply and clamps (RR-2026-010)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1/U2 at the SN 29500-2 reference value, 2 × 25 FIT (secondary quote); box discretes keep generic rates with their SN 29500 class named</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rows that stop actuation noted for SG-02 and SG-06 (DQ-362 A); their metric is the shared SG-01 estimate; no metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wire-end IDs of the WireViz drawings added; no rate, classification or metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format review: target as data, rate kind and wire ends as fields; no rate, classification or metric change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FMD-033 note: harness box SPICE pilot predictions per short path (PR #510); whole mode stays single-point; no rate, classification or metric change</t>
-  </si>
-  <si>
     <t xml:space="preserve">Camera-side termination R7/R8 added (FMD-C-014): one open latent, short single-point; total and SPF rates change</t>
   </si>
   <si>
+    <t xml:space="preserve">FMD-035 and FMD-036 linked to DFMEA DFM-022 and DFM-023 (DFMEA rev 0.13); no rate, classification or metric change</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mission profile</t>
   </si>
   <si>
@@ -880,7 +886,10 @@
     <t xml:space="preserve">One resistor open (camera side left with 120 Ω in intercept)</t>
   </si>
   <si>
-    <t xml:space="preserve">Latent: violates SG-009 only with the second resistor open (or the loopback open), which leaves the camera bus unterminated in intercept: the harness box SPICE pilot predicts a recessive edge of about 10.5 µs, missing the 1.5 µs sample point, so camera frames are lost while the device forwards (spice/predictions.md T-both-open, a prediction, no credit). One open alone leaves 120 Ω and an edge of about 0.06 µs. No check in the field; VS-HW-24 (e) measures both cases. Pass-through is not affected (R7/R8 sit on the NO side). No DFMEA row yet</t>
+    <t xml:space="preserve">DFM-022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latent: violates SG-009 only with the second resistor open (or the loopback open), which leaves the camera bus unterminated in intercept: the harness box SPICE pilot predicts a recessive edge of about 10.5 µs, missing the 1.5 µs sample point, so camera frames are lost while the device forwards (spice/predictions.md T-both-open, a prediction, no credit). One open alone leaves 120 Ω and an edge of about 0.06 µs. No check in the field; VS-HW-24 (e) measures both cases. Pass-through is not affected (R7/R8 sit on the NO side)</t>
   </si>
   <si>
     <t xml:space="preserve">FMD-036</t>
@@ -889,7 +898,10 @@
     <t xml:space="preserve">Short (camera CAN2_H to CAN2_L in intercept)</t>
   </si>
   <si>
-    <t xml:space="preserve">Camera bus held recessive in intercept: no camera frames reach the device, so stock PCS messages are not forwarded. RX checks cover car-side messages only (as FMD-017), so no mechanism is credited. Pass-through is not affected (R7/R8 sit on the NO side). No DFMEA row yet</t>
+    <t xml:space="preserve">DFM-023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camera bus held recessive in intercept: no camera frames reach the device, so stock PCS messages are not forwarded. RX checks cover car-side messages only (as FMD-017), so no mechanism is credited. Pass-through is not affected (R7/R8 sit on the NO side)</t>
   </si>
   <si>
     <t xml:space="preserve">FMD-023</t>
@@ -1674,30 +1686,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!O2:O37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
@@ -1711,7 +1723,7 @@
         <v>PASS</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -1745,33 +1757,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>7</v>
@@ -1817,7 +1829,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">07_SPFM_Calculation!D2</f>
@@ -1848,10 +1860,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>7</v>
@@ -1859,222 +1871,222 @@
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>333</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -2101,58 +2113,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>375</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -2171,7 +2183,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100"/>
@@ -2305,7 +2317,7 @@
     </row>
     <row r="10" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>46</v>
@@ -2314,7 +2326,21 @@
         <v>16</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2342,42 +2368,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2415,501 +2441,501 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>100</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L15" s="3"/>
     </row>
@@ -2943,136 +2969,136 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3103,87 +3129,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>40</v>
@@ -3193,19 +3219,19 @@
         <v>20</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="N2" s="3" t="n">
         <f aca="false">IF(D2="No",0,IF(AND(I2="No",J2="No"),H2,0))</f>
@@ -3228,31 +3254,31 @@
         <v>RF</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>5</v>
@@ -3262,10 +3288,10 @@
         <v>2.5</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="n">
@@ -3293,31 +3319,31 @@
         <v>SPF</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>55</v>
@@ -3327,10 +3353,10 @@
         <v>27.5</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="n">
@@ -3363,22 +3389,22 @@
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>80</v>
@@ -3388,19 +3414,19 @@
         <v>16</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="N5" s="3" t="n">
         <f aca="false">IF(D5="No",0,IF(AND(I5="No",J5="No"),H5,0))</f>
@@ -3423,29 +3449,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>10</v>
@@ -3455,19 +3481,19 @@
         <v>2</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L6" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="N6" s="3" t="n">
         <f aca="false">IF(D6="No",0,IF(AND(I6="No",J6="No"),H6,0))</f>
@@ -3490,29 +3516,29 @@
         <v>RF</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>10</v>
@@ -3522,19 +3548,19 @@
         <v>2</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L7" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="N7" s="3" t="n">
         <f aca="false">IF(D7="No",0,IF(AND(I7="No",J7="No"),H7,0))</f>
@@ -3557,31 +3583,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>90</v>
@@ -3591,19 +3617,19 @@
         <v>90</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="N8" s="3" t="n">
         <f aca="false">IF(D8="No",0,IF(AND(I8="No",J8="No"),H8,0))</f>
@@ -3626,29 +3652,29 @@
         <v>MPF_D</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>5</v>
@@ -3658,19 +3684,19 @@
         <v>5</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>90</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="N9" s="3" t="n">
         <f aca="false">IF(D9="No",0,IF(AND(I9="No",J9="No"),H9,0))</f>
@@ -3693,29 +3719,29 @@
         <v>RF</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>100</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>5</v>
@@ -3725,10 +3751,10 @@
         <v>5</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="n">
@@ -3756,31 +3782,31 @@
         <v>Safe</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>50</v>
@@ -3790,19 +3816,19 @@
         <v>5</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="L11" s="3" t="n">
         <v>99</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="N11" s="3" t="n">
         <f aca="false">IF(D11="No",0,IF(AND(I11="No",J11="No"),H11,0))</f>
@@ -3825,31 +3851,31 @@
         <v>MPF_D</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>10</v>
@@ -3859,10 +3885,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3" t="n">
@@ -3890,29 +3916,29 @@
         <v>SPF</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>40</v>
@@ -3922,10 +3948,10 @@
         <v>4</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K13" s="3"/>
       <c r="L13" s="3" t="n">
@@ -3953,29 +3979,29 @@
         <v>Safe</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>50</v>
@@ -3985,10 +4011,10 @@
         <v>7.5</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3" t="n">
@@ -4016,31 +4042,31 @@
         <v>Safe</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="T14" s="3"/>
       <c r="U14" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>30</v>
@@ -4050,19 +4076,19 @@
         <v>4.5</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>60</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="N15" s="3" t="n">
         <f aca="false">IF(D15="No",0,IF(AND(I15="No",J15="No"),H15,0))</f>
@@ -4085,31 +4111,31 @@
         <v>RF</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="T15" s="3"/>
       <c r="U15" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>20</v>
@@ -4119,10 +4145,10 @@
         <v>3</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K16" s="3"/>
       <c r="L16" s="3" t="n">
@@ -4150,29 +4176,29 @@
         <v>Safe</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>30</v>
@@ -4182,10 +4208,10 @@
         <v>6</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="n">
@@ -4213,31 +4239,31 @@
         <v>SPF</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T17" s="3"/>
       <c r="U17" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>30</v>
@@ -4247,10 +4273,10 @@
         <v>6</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="3" t="n">
@@ -4278,31 +4304,31 @@
         <v>SPF</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="T18" s="3"/>
       <c r="U18" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>40</v>
@@ -4312,10 +4338,10 @@
         <v>8</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3" t="n">
@@ -4348,22 +4374,22 @@
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>30</v>
@@ -4373,10 +4399,10 @@
         <v>15</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="3" t="n">
@@ -4404,31 +4430,31 @@
         <v>SPF</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="T20" s="3"/>
       <c r="U20" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>30</v>
@@ -4438,10 +4464,10 @@
         <v>15</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="3" t="n">
@@ -4469,31 +4495,31 @@
         <v>Safe</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T21" s="3"/>
       <c r="U21" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C22" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>40</v>
@@ -4503,10 +4529,10 @@
         <v>20</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="3" t="n">
@@ -4534,31 +4560,31 @@
         <v>SPF</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="T22" s="3"/>
       <c r="U22" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C23" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>50</v>
@@ -4568,10 +4594,10 @@
         <v>2.5</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="3" t="n">
@@ -4599,31 +4625,31 @@
         <v>SPF</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="T23" s="3"/>
       <c r="U23" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>50</v>
@@ -4633,10 +4659,10 @@
         <v>2.5</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="3" t="n">
@@ -4664,31 +4690,31 @@
         <v>Safe</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T24" s="3"/>
       <c r="U24" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>60</v>
@@ -4698,10 +4724,10 @@
         <v>0.24</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3" t="n">
@@ -4729,31 +4755,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="T25" s="3"/>
       <c r="U25" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>40</v>
@@ -4763,10 +4789,10 @@
         <v>0.16</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="3" t="n">
@@ -4794,31 +4820,31 @@
         <v>Safe</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T26" s="3"/>
       <c r="U26" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>40</v>
@@ -4828,10 +4854,10 @@
         <v>1.2</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3" t="n">
@@ -4859,31 +4885,31 @@
         <v>SPF</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="T27" s="3"/>
       <c r="U27" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>20</v>
@@ -4893,10 +4919,10 @@
         <v>0.6</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3" t="n">
@@ -4924,31 +4950,31 @@
         <v>SPF</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="T28" s="3"/>
       <c r="U28" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>40</v>
@@ -4958,10 +4984,10 @@
         <v>1.2</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="n">
@@ -4989,31 +5015,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="T29" s="3"/>
       <c r="U29" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>30</v>
@@ -5023,10 +5049,10 @@
         <v>0.6</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="n">
@@ -5054,31 +5080,31 @@
         <v>SPF</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="T30" s="3"/>
       <c r="U30" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>70</v>
@@ -5088,10 +5114,10 @@
         <v>1.4</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3" t="n">
@@ -5119,31 +5145,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="T31" s="3"/>
       <c r="U31" s="3" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C32" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>60</v>
@@ -5153,10 +5179,10 @@
         <v>0.24</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="3" t="n">
@@ -5183,30 +5209,32 @@
         <f aca="false">IF(D32="No","Safe",IF(I32="Yes",IF(L32=0,"SPF","RF"),IF(J32="Yes",IF(L32=0,"MPF_L","MPF_D"),"Safe")))</f>
         <v>MPF_L</v>
       </c>
-      <c r="S32" s="3"/>
+      <c r="S32" s="3" t="s">
+        <v>284</v>
+      </c>
       <c r="T32" s="3"/>
       <c r="U32" s="3" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C33" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>40</v>
@@ -5216,10 +5244,10 @@
         <v>0.16</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="3" t="n">
@@ -5246,30 +5274,32 @@
         <f aca="false">IF(D33="No","Safe",IF(I33="Yes",IF(L33=0,"SPF","RF"),IF(J33="Yes",IF(L33=0,"MPF_L","MPF_D"),"Safe")))</f>
         <v>SPF</v>
       </c>
-      <c r="S33" s="3"/>
+      <c r="S33" s="3" t="s">
+        <v>288</v>
+      </c>
       <c r="T33" s="3"/>
       <c r="U33" s="3" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>30</v>
@@ -5279,10 +5309,10 @@
         <v>3</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3" t="n">
@@ -5310,31 +5340,31 @@
         <v>SPF</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="T34" s="3"/>
       <c r="U34" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>70</v>
@@ -5344,10 +5374,10 @@
         <v>7</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3" t="n">
@@ -5375,31 +5405,31 @@
         <v>Safe</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="T35" s="3"/>
       <c r="U35" s="3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C36" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>50</v>
@@ -5409,10 +5439,10 @@
         <v>1</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3" t="n">
@@ -5440,31 +5470,31 @@
         <v>MPF_L</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="T36" s="3"/>
       <c r="U36" s="3" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G37" s="3" t="n">
         <v>50</v>
@@ -5474,10 +5504,10 @@
         <v>1</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3" t="n">
@@ -5505,11 +5535,11 @@
         <v>Safe</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="T37" s="3"/>
       <c r="U37" s="3" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -5536,57 +5566,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -5616,22 +5646,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5639,10 +5669,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!O2:O37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$M$2:$M$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$E$2:$E$2))+SUM(06_FMEDA_Worksheet!P2:P37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$N$2:$N$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$F$2:$F$2))</f>
@@ -5691,22 +5721,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>315</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>316</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>311</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>7</v>
@@ -5714,10 +5744,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">SUM(06_FMEDA_Worksheet!Q2:Q37)+(SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$O$2:$O$2)-SUMIF(06b_Per_Goal_Rows!$A$2:$A$2,"SG-07",06b_Per_Goal_Rows!$G$2:$G$2))</f>

</xml_diff>